<commit_message>
Update Intermediate sheet docs: pw_* arrays now Excel-loaded, noIS deleted
- Rows 23-24: updated description from 'Hard-coded' to 'READ FROM EXCEL
  Materials col W/X'; updated values to current 6-material arrays
- Row 25: noIS arrays marked as DELETED 2026-04-22 with rationale
- Row 22: section header refreshed with new date
- Sources clarified as [ASSUMED+LIT] with Gadaleta/Verma/Schmutz citations

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/22APRIL.xlsx
+++ b/22APRIL.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00000"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* \-??_-;_-@_-"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -211,8 +211,12 @@
       <b val="1"/>
       <color rgb="001F497D"/>
     </font>
+    <font>
+      <strike val="1"/>
+      <color rgb="FF808080"/>
+    </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -328,6 +332,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -495,7 +504,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -707,6 +716,7 @@
     <xf numFmtId="0" fontId="27" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -10319,8 +10329,8 @@
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A9:A11"/>
     <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A1:B1"/>
     <mergeCell ref="B3:B5"/>
-    <mergeCell ref="A1:B1"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A18:A20"/>
   </mergeCells>
@@ -11296,7 +11306,7 @@
     <row r="22">
       <c r="A22" s="76" t="inlineStr">
         <is>
-          <t>── Process Waste Fate &amp; NoIS Disposal Arrays (Consensus-validated 2026-04-02) ──</t>
+          <t>── Process Waste Fate Arrays (Consensus-validated 2026-04-22) ──</t>
         </is>
       </c>
     </row>
@@ -11308,22 +11318,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>[0.70, 0.80, 0.85, 0.50, 0.85]</t>
+          <t>Materials sheet col W (rows 3-8)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>fraction [PLASTIC/PAPER/Fe/TEXTILE/NFe]</t>
+          <t>fraction [PLASTIC/PAPER/Fe/TEXTILE/NFe/ORGANIC]</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Hard-coded in ALP Main (not read from Excel). Recycling residue → landfill per material.</t>
+          <t>READ FROM EXCEL — Materials sheet col W (23). Values: {0.74, 0.89, 0.94, 0.56, 0.89, 0.86}. Loaded at startup via getCellNumericValue("Materials", row, 23). Used by BOTH IS and noIS code paths (unified since 2026-04-22). Process waste (recycling residue) fraction → sanitary landfill, per material. [ASSUMED] based on physical combustibility rationale + SE Asia disposal patterns. LF+Incin=1.0 per material (sum_check col Y confirms).</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>[LIT] Vietnam ET Journal 2024; SE Asia MSW 2023 (Sustainability); Thai Al LCA 2025 (IOP); Energies 2024 (Textile)</t>
+          <t>[ASSUMED+LIT] Landfill-dominant regime: Gadaleta et al. (2023) Sustainability; Verma et al. (2016) HCMC MSW; Noudeng et al. (2024). Metals inert → landfill: Agamuthu &amp; Babel (2023). No direct quantitative data for industrial process waste splits in Vietnam — values are modelling assumptions calibrated to literature patterns. Document as [ASSUMED] in Appendix X.</t>
         </is>
       </c>
     </row>
@@ -11335,49 +11345,49 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>[0.25, 0.10, 0.05, 0.40, 0.10]</t>
+          <t>Materials sheet col X (rows 3-8)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>fraction [PLASTIC/PAPER/Fe/TEXTILE/NFe]</t>
+          <t>fraction [PLASTIC/PAPER/Fe/TEXTILE/NFe/ORGANIC]</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Hard-coded in ALP Main (not read from Excel). Recycling residue → incineration per material.</t>
+          <t>READ FROM EXCEL — Materials sheet col X (24). Values: {0.26, 0.11, 0.06, 0.44, 0.11, 0.14}. Complement of pw_landfillSharePerMat (LF+Incin=1.0). Process waste fraction routed to combustion → ash → bricks. Higher share for combustible materials (PLASTIC[0]=0.26, TEXTILE[3]=0.44); lower for inert metals (FERROUS[2]=0.06, NON_FERROUS[4]=0.11).</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>[LIT] SE Asia open burning (ES&amp;T 2020); Energies 2024; Thai Al 2025; HCMC MSW 2016</t>
+          <t>[ASSUMED+LIT] Combustible fractions: Schmutz &amp; Som (2022) Resources Conserv Recycl — Swiss textile waste 37% incinerated; Nguyen et al. (2024) RSC Advances — incineration primary method for mixed industrial waste northern Vietnam. Metals low incin share: inert/non-combustible, mostly landfilled if disposed (Agamuthu &amp; Babel 2023). Values [ASSUMED] — no SE Asia industrial process waste split data available in literature (confirmed by Consensus search 2026-04-22).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="76" t="inlineStr">
-        <is>
-          <t>noIS_landfillShare[] / noIS_incinerationShare[]</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>LF:[0.70,0.80,0.15,0.55,0.15] / IN:[0.25,0.10,0.05,0.35,0.05]</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>fraction [PLASTIC/PAPER/Fe/TEXTILE/NFe]</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>BAU disposal (useIS=false). Hard-coded in ALP Main. [0],[1] PLASTIC/PAPER aligned to pw_* arrays — modeling assumption subject to sensitivity analysis [ASSUMED]. [2],[4] FERROUS/NON_FERROUS low shares reflect informal scrap dealer diversion (Wilson et al. 2006; Nguyen et al. 2019) [LIT].</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>[LIT] Vietnam TV MFA 2018 (RCR, metals); HCMC MSW 2016; Vietnam plastic 2024; Energies 2024; Thai Al LCA 2025</t>
+      <c r="A25" s="87" t="inlineStr">
+        <is>
+          <t>noIS_landfillShare[] / noIS_incinerationShare[] — DELETED 2026-04-22</t>
+        </is>
+      </c>
+      <c r="B25" s="87" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C25" s="87" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="D25" s="87" t="inlineStr">
+        <is>
+          <t>Arrays deleted 2026-04-22. Both IS and noIS code paths now use pw_landfillSharePerMat[] and pw_incinerationSharePerMat[] from Materials col W/X. Rationale: process waste split fractions are the same regardless of IS mode — the difference between IS and noIS is the VOLUME reaching combustion, not the split ratios.</t>
+        </is>
+      </c>
+      <c r="E25" s="87" t="inlineStr">
+        <is>
+          <t>See git commit 37aa11c</t>
         </is>
       </c>
     </row>

</xml_diff>